<commit_message>
updated code to handle latency for getting applications in datatable
</commit_message>
<xml_diff>
--- a/Data/Input/Manager Matrix.xlsx
+++ b/Data/Input/Manager Matrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HarikaMalyala\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft3346595-my.sharepoint.com/personal/abhi_khandavalli_ashlingpartners_com/Documents/Desktop/Dominium/02_20_DuProdDeploy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B23A0CF-1928-4273-9D6F-959E95CC86C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{41C4F52D-CCC3-496E-9301-18879BC5D867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{06A0A5C0-A0A5-454D-B5C2-7A6641829BD3}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17448" windowHeight="9876" xr2:uid="{06A0A5C0-A0A5-454D-B5C2-7A6641829BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
   <si>
     <t>State</t>
   </si>
@@ -45,6 +45,45 @@
   </si>
   <si>
     <t>File Reviewer</t>
+  </si>
+  <si>
+    <t>67 Flats</t>
+  </si>
+  <si>
+    <t>Aviara Flats</t>
+  </si>
+  <si>
+    <t>Vista Ridge</t>
+  </si>
+  <si>
+    <t>AZ</t>
+  </si>
+  <si>
+    <t>Copper Cove</t>
+  </si>
+  <si>
+    <t>Solstice of Mesa</t>
+  </si>
+  <si>
+    <t>Estrella Springs at Canyon Trails</t>
+  </si>
+  <si>
+    <t>Suncrest Vista at Canyon Trails</t>
+  </si>
+  <si>
+    <t>Casa Azure</t>
+  </si>
+  <si>
+    <t>The Safford</t>
+  </si>
+  <si>
+    <t>Juniper Square</t>
+  </si>
+  <si>
+    <t>Cholla Ranch</t>
+  </si>
+  <si>
+    <t>Kate Holmes</t>
   </si>
 </sst>
 </file>
@@ -416,14 +455,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E663267-87A7-4CC2-A0CC-65D38C2609EB}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="44.7109375" customWidth="1"/>
+    <col min="2" max="2" width="44.6640625" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -432,6 +471,132 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -748,6 +913,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7589ac45-c6d7-49c5-afa1-0d2a3e0f973c">
@@ -763,15 +937,6 @@
     <_Flow_SignoffStatus xmlns="7589ac45-c6d7-49c5-afa1-0d2a3e0f973c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -795,6 +960,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69FB3FBB-EEE5-40B6-9E3A-01D738F323B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB0AEC57-6438-4C64-BA9D-C279A2954843}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -804,12 +977,4 @@
     <ds:schemaRef ds:uri="92efdeaa-2ae3-407c-a5b8-d7c39eaf4b0f"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69FB3FBB-EEE5-40B6-9E3A-01D738F323B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>